<commit_message>
Add scatter chart comparing Tiempo (x) vs Velocidad (y); injected chart XML directly to preserve cached values
</commit_message>
<xml_diff>
--- a/Libro1.xlsx
+++ b/Libro1.xlsx
@@ -98,6 +98,1000 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:t>Tiempo vs Velocidad</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Hoja1!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Velocidad</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Hoja1!$A$2:$A$138</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="137"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>8</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>26</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>27</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>31</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>32</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>42</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>43</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>46</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>48</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>53</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>55</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>56</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>62</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>64</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>65</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>66</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>67</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>68</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>71</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>77</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>78</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>81</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>82</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>88</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>89</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>92</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>95</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>96</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>98</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>104</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>105</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>109</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>111</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>112</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>123</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>125</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>126</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>129</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>130</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>133</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>136</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>137</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Hoja1!$B$2:$B$138</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="137"/>
+                <c:pt idx="0">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>33</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>28</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>30</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>29</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>34</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>36</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>37</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>39</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>41</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>38</c:v>
+                </c:pt>
+                <c:pt idx="34">
+                  <c:v>45</c:v>
+                </c:pt>
+                <c:pt idx="35">
+                  <c:v>40</c:v>
+                </c:pt>
+                <c:pt idx="36">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="37">
+                  <c:v>49</c:v>
+                </c:pt>
+                <c:pt idx="38">
+                  <c:v>44</c:v>
+                </c:pt>
+                <c:pt idx="39">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="40">
+                  <c:v>47</c:v>
+                </c:pt>
+                <c:pt idx="41">
+                  <c:v>50</c:v>
+                </c:pt>
+                <c:pt idx="42">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="43">
+                  <c:v>52</c:v>
+                </c:pt>
+                <c:pt idx="44">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="45">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="46">
+                  <c:v>53</c:v>
+                </c:pt>
+                <c:pt idx="47">
+                  <c:v>57</c:v>
+                </c:pt>
+                <c:pt idx="48">
+                  <c:v>51</c:v>
+                </c:pt>
+                <c:pt idx="49">
+                  <c:v>58</c:v>
+                </c:pt>
+                <c:pt idx="50">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="51">
+                  <c:v>54</c:v>
+                </c:pt>
+                <c:pt idx="52">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="53">
+                  <c:v>59</c:v>
+                </c:pt>
+                <c:pt idx="54">
+                  <c:v>60</c:v>
+                </c:pt>
+                <c:pt idx="55">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="56">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="57">
+                  <c:v>61</c:v>
+                </c:pt>
+                <c:pt idx="58">
+                  <c:v>69</c:v>
+                </c:pt>
+                <c:pt idx="59">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="60">
+                  <c:v>63</c:v>
+                </c:pt>
+                <c:pt idx="61">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="62">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="63">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="64">
+                  <c:v>70</c:v>
+                </c:pt>
+                <c:pt idx="65">
+                  <c:v>72</c:v>
+                </c:pt>
+                <c:pt idx="66">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="67">
+                  <c:v>73</c:v>
+                </c:pt>
+                <c:pt idx="68">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="69">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="70">
+                  <c:v>80</c:v>
+                </c:pt>
+                <c:pt idx="71">
+                  <c:v>74</c:v>
+                </c:pt>
+                <c:pt idx="72">
+                  <c:v>75</c:v>
+                </c:pt>
+                <c:pt idx="73">
+                  <c:v>76</c:v>
+                </c:pt>
+                <c:pt idx="74">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="75">
+                  <c:v>79</c:v>
+                </c:pt>
+                <c:pt idx="76">
+                  <c:v>85</c:v>
+                </c:pt>
+                <c:pt idx="77">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="78">
+                  <c:v>87</c:v>
+                </c:pt>
+                <c:pt idx="79">
+                  <c:v>83</c:v>
+                </c:pt>
+                <c:pt idx="80">
+                  <c:v>84</c:v>
+                </c:pt>
+                <c:pt idx="81">
+                  <c:v>90</c:v>
+                </c:pt>
+                <c:pt idx="82">
+                  <c:v>86</c:v>
+                </c:pt>
+                <c:pt idx="83">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="84">
+                  <c:v>94</c:v>
+                </c:pt>
+                <c:pt idx="85">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="86">
+                  <c:v>97</c:v>
+                </c:pt>
+                <c:pt idx="87">
+                  <c:v>91</c:v>
+                </c:pt>
+                <c:pt idx="88">
+                  <c:v>93</c:v>
+                </c:pt>
+                <c:pt idx="89">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="90">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="91">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="92">
+                  <c:v>102</c:v>
+                </c:pt>
+                <c:pt idx="93">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="94">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="95">
+                  <c:v>107</c:v>
+                </c:pt>
+                <c:pt idx="96">
+                  <c:v>99</c:v>
+                </c:pt>
+                <c:pt idx="97">
+                  <c:v>106</c:v>
+                </c:pt>
+                <c:pt idx="98">
+                  <c:v>101</c:v>
+                </c:pt>
+                <c:pt idx="99">
+                  <c:v>108</c:v>
+                </c:pt>
+                <c:pt idx="100">
+                  <c:v>103</c:v>
+                </c:pt>
+                <c:pt idx="101">
+                  <c:v>110</c:v>
+                </c:pt>
+                <c:pt idx="102">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="103">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="104">
+                  <c:v>115</c:v>
+                </c:pt>
+                <c:pt idx="105">
+                  <c:v>116</c:v>
+                </c:pt>
+                <c:pt idx="106">
+                  <c:v>113</c:v>
+                </c:pt>
+                <c:pt idx="107">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="108">
+                  <c:v>120</c:v>
+                </c:pt>
+                <c:pt idx="109">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="110">
+                  <c:v>114</c:v>
+                </c:pt>
+                <c:pt idx="111">
+                  <c:v>119</c:v>
+                </c:pt>
+                <c:pt idx="112">
+                  <c:v>117</c:v>
+                </c:pt>
+                <c:pt idx="113">
+                  <c:v>118</c:v>
+                </c:pt>
+                <c:pt idx="114">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="115">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="116">
+                  <c:v>121</c:v>
+                </c:pt>
+                <c:pt idx="117">
+                  <c:v>122</c:v>
+                </c:pt>
+                <c:pt idx="118">
+                  <c:v>124</c:v>
+                </c:pt>
+                <c:pt idx="119">
+                  <c:v>127</c:v>
+                </c:pt>
+                <c:pt idx="120">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="121">
+                  <c:v>128</c:v>
+                </c:pt>
+                <c:pt idx="122">
+                  <c:v>131</c:v>
+                </c:pt>
+                <c:pt idx="123">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="124">
+                  <c:v>136</c:v>
+                </c:pt>
+                <c:pt idx="125">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="126">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="127">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="128">
+                  <c:v>134</c:v>
+                </c:pt>
+                <c:pt idx="129">
+                  <c:v>132</c:v>
+                </c:pt>
+                <c:pt idx="130">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="131">
+                  <c:v>135</c:v>
+                </c:pt>
+                <c:pt idx="132">
+                  <c:v>143</c:v>
+                </c:pt>
+                <c:pt idx="133">
+                  <c:v>141</c:v>
+                </c:pt>
+                <c:pt idx="134">
+                  <c:v>137</c:v>
+                </c:pt>
+                <c:pt idx="135">
+                  <c:v>139</c:v>
+                </c:pt>
+                <c:pt idx="136">
+                  <c:v>147</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="111111111"/>
+        <c:axId val="222222222"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="111111111"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:t>Tiempo</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:crossAx val="222222222"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="222222222"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:t>Velocidad</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+        </c:title>
+        <c:majorGridlines/>
+        <c:crossAx val="111111111"/>
+        <c:crosses val="autoZero"/>
+      </c:valAx>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:overlay val="0"/>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1671,5 +2665,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>